<commit_message>
Update DRM and BOQ Format
</commit_message>
<xml_diff>
--- a/data/template/drm/Template_DRM_Report.xlsx
+++ b/data/template/drm/Template_DRM_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JACOBS\SERVICE\API\data\template\drm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF38CCE4-9E23-41A5-88AE-1BEE63B1ACE8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB5EE854-59B5-46C9-BE74-3258471648CB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -231,7 +231,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -263,19 +263,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -307,6 +338,21 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -830,55 +876,55 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="6" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" style="3" customWidth="1"/>
-    <col min="3" max="4" width="33.28515625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25" style="3" customWidth="1"/>
-    <col min="8" max="8" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9" style="3"/>
-    <col min="10" max="10" width="19.140625" style="3" customWidth="1"/>
-    <col min="11" max="14" width="9" style="3"/>
-    <col min="15" max="15" width="11.5703125" style="3" customWidth="1"/>
-    <col min="16" max="16384" width="9" style="3"/>
+    <col min="1" max="1" width="5.7109375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" style="1" customWidth="1"/>
+    <col min="3" max="4" width="33.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9" style="1"/>
+    <col min="10" max="10" width="19.140625" style="1" customWidth="1"/>
+    <col min="11" max="14" width="9" style="1"/>
+    <col min="15" max="15" width="11.5703125" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="31.5" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" ht="15">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="8" t="s">
         <v>5</v>
       </c>
     </row>
@@ -900,128 +946,128 @@
   <dimension ref="A1:S3"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" style="6" customWidth="1"/>
-    <col min="5" max="5" width="22.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.7109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.5703125" style="7" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.7109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="28.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.140625" style="8" customWidth="1"/>
-    <col min="20" max="16384" width="9" style="3"/>
+    <col min="1" max="1" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="28.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.140625" style="6" customWidth="1"/>
+    <col min="20" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
     </row>
     <row r="2" spans="1:19" ht="21" customHeight="1">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2"/>
-      <c r="S2" s="2"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="14"/>
+      <c r="Q2" s="14"/>
+      <c r="R2" s="14"/>
+      <c r="S2" s="14"/>
     </row>
     <row r="3" spans="1:19" ht="22.5">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="L3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="N3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="O3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="P3" s="4" t="s">
+      <c r="P3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="Q3" s="4" t="s">
+      <c r="Q3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="R3" s="4" t="s">
+      <c r="R3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="S3" s="5" t="s">
+      <c r="S3" s="3" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1043,112 +1089,112 @@
   <dimension ref="A1:T2"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="35.140625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="23.7109375" style="11" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" style="3" customWidth="1"/>
-    <col min="9" max="9" width="29.7109375" style="3" customWidth="1"/>
-    <col min="10" max="10" width="17" style="3" customWidth="1"/>
-    <col min="11" max="11" width="13.28515625" style="3" customWidth="1"/>
-    <col min="12" max="12" width="23.7109375" style="3" customWidth="1"/>
-    <col min="13" max="13" width="25" style="3" customWidth="1"/>
-    <col min="14" max="14" width="16.140625" style="3" customWidth="1"/>
-    <col min="15" max="15" width="18.140625" style="3" customWidth="1"/>
-    <col min="16" max="16" width="15.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.42578125" style="3" customWidth="1"/>
-    <col min="19" max="19" width="28.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.5703125" style="6" customWidth="1"/>
-    <col min="21" max="16384" width="8.5703125" style="3"/>
+    <col min="1" max="1" width="9.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="35.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" style="9" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="29.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="17" style="1" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="23.7109375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="25" style="1" customWidth="1"/>
+    <col min="16" max="16" width="16.140625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.42578125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="28.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.5703125" style="4" customWidth="1"/>
+    <col min="21" max="16384" width="8.5703125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="3" customFormat="1" ht="45" customHeight="1">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:20" ht="45" customHeight="1">
+      <c r="A1" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
-      <c r="T1" s="2"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="16"/>
+      <c r="T1" s="17"/>
     </row>
-    <row r="2" spans="1:20" s="3" customFormat="1" ht="15">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:20" ht="15">
+      <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="K2" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="J2" s="12" t="s">
+      <c r="L2" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="K2" s="14" t="s">
+      <c r="M2" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="L2" s="12" t="s">
+      <c r="N2" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M2" s="12" t="s">
+      <c r="O2" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="P2" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="O2" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="P2" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q2" s="12" t="s">
+      <c r="Q2" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="R2" s="12" t="s">
+      <c r="R2" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="S2" s="12" t="s">
+      <c r="S2" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="T2" s="12" t="s">
+      <c r="T2" s="10" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>